<commit_message>
Covid form medic (#76) (#82)
* Covid form medic (#76)

* added app_settings (#78)

Co-authored-by: nKataraia <55187908+nKataraia@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/forms/app/covid_education.xlsx
+++ b/forms/app/covid_education.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20377"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A47927-73B3-4D80-9373-690439AAA7F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
     <sheet name="choices" sheetId="2" r:id="rId2"/>
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="197">
   <si>
     <t>type</t>
   </si>
@@ -176,624 +177,31 @@
     <t>covid19_intro_note</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;As a CHV, you are responsible for making sure that you are providing the community with health education and services while trying to take precautions to stop the transmission of Coronavirus to one another. Therefore, make sure you consider the following while you conduct the visits:  
-•       All visits must be conducted outside the home in open space, where there is air flow and risk of spread of disease is less.
-•       You must wear a cloth mask when conducting home visits and moving through the community. If you do not have a mask, please do not make the household visit.
-•        Wash your hands with soap/sanitizer as many time as you can while at home, once you are at the client’s house and when you leave.
-•        Keep a 2 meters distance while talking to your clients.
-•        Don’t shake hands with your clients. 
-•        Avoid group gatherings.
-•        Cover your mouth with a towel or elbow when you sneeze or cough. 
-•        Do not go for a visit if you have symptoms of fever, cough or frequent sneezing.&lt;/span&gt; 
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;Kama mhudumu wa afya ya jamii, una jukumu la kuhakikisha unatoa elimu ya afya ya jamii na huduma huku ukijikinga ili kuepusha kusambaa kwa maambukizi ya korona kutoka kwa mtu mmoja kwenda kwa mwengine. Hivyo hakikisha unazingatia yafuatayo wakati ukiwa unatoa huduma:
-•         Matembeleo yote yafanye nje ya nyumba kwenye eneo la wazi, ambapo kuna mzunguko wa hewa kwa kupunguza athari za kuenea kwa maambukizi.
-•         Ni Lazima kuvaa barakoa yako muda wote unafanya matembeleo au kutembea kwenye jamii. Kama huna barakoa, tafadhali acha kufanya matembeleo.
-•        Osha mikono yako kwa maji na sabuni au kutumia vitakasa mikono mara nyingi kadiri unavyoweza ukiwa nyumbani kwako,nyumbani kwa mteja wako na pindi ukimaliza kutoa huduma. 
-•        Hakikisha kuna umbali wa mita mbili kati yako na mteja wako unayeenda kumtembelea 
-•        Pindi ukiongea na wateja wako , usishikane mikono. 
-•        Epuka mikusanyiko. 
-•        Funika mdomo wako kwa kitambaa au kiwiko unavyooenda chafya au kukohoa. 
-•        Tafadhali usiende kutoa huduma ukijihisi na dalili za homa na kukohoa na kwenda chafya kwa wingi.&lt;/span&gt; 
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">end group </t>
-  </si>
-  <si>
-    <t>introductory_qns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduction to COVID </t>
-  </si>
-  <si>
-    <t>Muhtasari</t>
   </si>
   <si>
     <t>field-list</t>
   </si>
   <si>
-    <t>introduction</t>
-  </si>
-  <si>
-    <t>Hi, how are you? Today before we start our visit, please let’s talk a little about the coronavirus. As we know the world is now experiencing this tragedy of coronavirus and we as Zanzibarians have the disease here as well and the infection is affecting people, and it is our responsibility to protect ourselves</t>
-  </si>
-  <si>
-    <t>Habari yako, leo kabla hatujaanza tembeleo letu naomba tuzungumzie kidogo kuhusu virusi vya Korona. Kama tunavyojua dunia sasa inakabiliwa na janga hili la virusi vya Korona na sisi kama wanzanzibar huu ugonjwa umeshafika na teyari unawaathiri watu, na ni jukumu letu sote kujilinda.</t>
-  </si>
-  <si>
     <t>select_one yes_no</t>
-  </si>
-  <si>
-    <t>corona_awareness</t>
-  </si>
-  <si>
-    <t>Do you know anything about this disease?</t>
-  </si>
-  <si>
-    <t>Je unafahamu chochote kuhusu ugonjwa huu?</t>
   </si>
   <si>
     <t>yes</t>
   </si>
   <si>
-    <t>listen_to_mother</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Listen to the mother talking about coronavirus and add to this description.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Msikilize mama akiongea kuhusu ugonjwa wa korona na baadae ongezea maelezo haya.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>selected(${corona_awareness},"yes")</t>
-  </si>
-  <si>
-    <t>qns_from_family</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before we start, do the householders have something specific about the Coronavirus they want to know or tell me? </t>
-  </si>
-  <si>
-    <t>Kabla hatujaanza ,Je wanakaya wana jambo mahsusi kuhusu Korona wanalotaka kujua au kuniambia?</t>
-  </si>
-  <si>
-    <t>answer_questions</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Answer if you can, otherwise call 190.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Jibu ikiwa unaweza, vinginevyo piga simu ya 190.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>selected(${qns_from_family},"yes")</t>
-  </si>
-  <si>
-    <t>msg_for_chv_questions</t>
-  </si>
-  <si>
-    <t>&lt;span style="display:block;color:red;font-style: italic;padding-left:1em"&gt;Don't read aloud. Fill in yourself. (CHV). &lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:red;font-style: italic"&gt;Usimsomee, jaza wewe (CHV). &lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>select_multiple asked_qns</t>
-  </si>
-  <si>
     <t>asked_qns</t>
-  </si>
-  <si>
-    <t>Select all the questions which were asked by the client</t>
-  </si>
-  <si>
-    <t>Chagua masuali yote yalioulizwa na mteja.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes </t>
-  </si>
-  <si>
-    <t>msg_for_chv_other_qn</t>
-  </si>
-  <si>
-    <t>selected(${asked_qns},"none")</t>
   </si>
   <si>
     <t>text</t>
   </si>
   <si>
-    <t>other_question</t>
-  </si>
-  <si>
-    <t>Please list the asked questions</t>
-  </si>
-  <si>
-    <t>Tafadhali taja masuali yalioulizwa.</t>
-  </si>
-  <si>
-    <t>intro_to_corona</t>
-  </si>
-  <si>
-    <t>What is Coronavirus disease?</t>
-  </si>
-  <si>
-    <t>Ugonjwa wa  Korona ni nini?</t>
-  </si>
-  <si>
-    <t>what_is_corona</t>
-  </si>
-  <si>
-    <t>It is a viral disease caused by a new kind of Coronavirus, which is transmitted from one infected person to another. There are other coronaviruses that cause the flu, but this one is new and worse than the others.</t>
-  </si>
-  <si>
-    <t>Huu ni ugonjwa unaosababishwa na virusi vipya vya korona, ugonjwa huu unasambaa kutoka kwa mtu mmoja kwenda kwa mwengine, Kuna aina nyengine za virusi vya korona ambavyo husababisha mafua, lakini hibhivi i ni virusi vipya na hatari Zaidi kusambaa.</t>
-  </si>
-  <si>
     <t>corona_transmission</t>
-  </si>
-  <si>
-    <t>How is Corona disease transmitted?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ugonjwa wa Korona unaambukizwa vipi? </t>
-  </si>
-  <si>
-    <t>how_is_it_transmitted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• This disease is transmitted by airborne fluids when a person sneezes, coughs, talks and breathes.
-• A person can also get infections by touching infected objects and then touching their eyes, nose or mouth before washing their hands with soapy water.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ugonjwa huu huenea kwa  majimaji yenye maambukizi yatokayo njia ya hewa pale mtu anapopiga chafya,  kukohoa, kusema na kupenga mafua.
-• Pia mtu anaweza kupata maambukizi kwa kugusa vitu vyenye maambukizi ya ugonjwa huo na baadae akagusa macho, pua au mdomo kabla ya kunawa mikono yake kwa maji ya kutiririka na sabuni.
-</t>
   </si>
   <si>
     <t>corona_symptoms</t>
   </si>
   <si>
-    <t>What are the symptoms of Corona disease?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ni zipi dalili za ugonjwa wa Korona? </t>
-  </si>
-  <si>
-    <t>what_are_corona_symptoms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-• A corona patient may take 1 to 14 days to show symptoms or signs.
-• Symptoms and signs of the disease include:
-     1.To get a high fever
-     2.Coughing
-     3.Trouble breathing
-     4.Sneezing frequently
-     5.Acquiring severe flu
-     6.Headache
-     7.Sore throat and
-     8.Not tasting or smelling
-•These symptoms are not unique, They may have other symptoms, Please contact a health professional / get to the center for more symptoms or if the condition worsens.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•   Mgonjwa wa Korona anaweza kuchukua siku moja hadi kumi na nne (1-14) kuweza kuonesha dalili au ishara. 
-•  Dalili na ishara za ugonjwa huo ni pamoja na:
-        1. Kupata homa kali 
-        2. Kukohoa 
-        3. Kupumua kwa shida
-        4. Chafya za mara kwa mara 
-        5. Kupata mafua makali 
-        6. Kuumwa na kichwa 
-        7. Vidonda vya koo na 
-        8. Kutohisi ladha ya chakula au kutosikia harufu
-•   Dalili hizi sio za kipekee, Inaweza kuwa na dalili nyengine zaidi, Tafadhali wasiliana na mtaalamu wa afya/ fika kituoni kwa dalili  zaidi au ukiona hali inazidi kuwa mbaya.
-</t>
-  </si>
-  <si>
-    <t>has_corona</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Does anyone in this household have any of the symptoms mentioned?</t>
-  </si>
-  <si>
-    <t>Je kuna Mtu yeyote kwenye kaya hii ana dalili hizi tulizozitaja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">report_client </t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;If the client has any of the above symptoms, please report this to the district surveillance officer immediately.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Ikiwa mteja ana dalili zozote kati ya hizi, tafadhali toa ripoti kwa Afisa uchunguzi wa wilaya kwa haraka.&lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>selected(${has_corona},"yes")</t>
-  </si>
-  <si>
-    <t>sneezing</t>
-  </si>
-  <si>
-    <t>sneezing.png</t>
-  </si>
-  <si>
-    <t>coughing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coughing.png </t>
-  </si>
-  <si>
-    <t>headache</t>
-  </si>
-  <si>
-    <t>headache.png</t>
-  </si>
-  <si>
-    <t>corona_prevention</t>
-  </si>
-  <si>
-    <t>How will you protect yourself from Coronavirus?</t>
-  </si>
-  <si>
-    <t>Vipi utajikinga na ugonjwa wa Korona?</t>
-  </si>
-  <si>
-    <t>how_to_prevent_corona</t>
-  </si>
-  <si>
-    <t>• Wash hands with clean running water and regular soap (at least 20 seconds)
-• Avoid sitting in public gatherings and stay at a distance of one meter
-• Cover the mouth and nose with a towel, tissue or elbow when sneezing, coughing or flushing the flu
-• Avoid handshaking
-• Avoid touching your mouth, nose and eyes before washing your hands
-• Avoid unnecessary trips
-• Remember to wash hands with soap and running water before entering the home
-• Remember to wear a mask whenever you step out of your house.</t>
-  </si>
-  <si>
-    <t>•  Nawa mikono kwa  maji safi ya kutiririka na sabuni mara kwa mara(angalau kwa sekunde 20) (Wafundishe kutengeneza kibuyu chirizi kama hamna mferji)
-•  Epuka kukaa kwenye mikusanyiko ya watu na ukae umbali wa mita moja 
-•  Funika mdomo na pua kwa kitambaa, tishu au kiwiko cha mkono unapopiga chafya, kukohoa au kupenga mafua
-•  Epuka tabia ya  kupeana mikono
-•  Epuka kushika  mdomo, pua na macho kabla ya kuosha mikono
-•  Epuka safari zisizo za lazima
-•  Kumbuka kuosha mikono kwa sababuni na maji tiririka muda wote kabla ya kuingia nyumbani
-•  Kumbuka Kuvaa barakoa muda wote unapotoka nje ya nyumba yako.</t>
-  </si>
-  <si>
-    <t>hand_washing</t>
-  </si>
-  <si>
-    <t>hand_washing.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no_gathering </t>
-  </si>
-  <si>
-    <t>no_gathering.png</t>
-  </si>
-  <si>
-    <t>elbow_cough</t>
-  </si>
-  <si>
-    <t>elbow_cough.png</t>
-  </si>
-  <si>
-    <t>no_handshake</t>
-  </si>
-  <si>
-    <t>no_handshake.png</t>
-  </si>
-  <si>
-    <t>no_face_touch</t>
-  </si>
-  <si>
-    <t>no_face_touch.png</t>
-  </si>
-  <si>
-    <t>no_travel</t>
-  </si>
-  <si>
-    <t>no_travel.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">corona_prevention </t>
-  </si>
-  <si>
-    <t>additional_guidelines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Additional Guidelines </t>
-  </si>
-  <si>
-    <t>Maelezo Muhimu kuhusu Corona</t>
-  </si>
-  <si>
-    <t>list_of_guidelines</t>
-  </si>
-  <si>
-    <t>• Recognize that a person with a coronavirus infection can infect another person even if they have not begun to show signs and symptoms of the disease.
-•  Report promptly to community health workers (CHV) if there is a resident or you have received a visitor with symptoms of a coronavirus 
-•  Coronavirus currently has no cure or vaccine and is rapidly spreading around the world.
-•  You have a responsibility to protect yourself and others
-•  When you feel any signs or symptoms of severe cold flu stay at home and call by phone. Call at no cost: 190
-•  Also let them know about the Facebook, insta and whats apps of the health education unit of the Ministry of Health so that you can find more factual information and trends and events in the Zanzibar coronavirus epidemic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-• Tambua kuwa mtu mwenye virusi vya ugonjwa wa Korona anaweza kumuambukiza mtu mwengine hata kama hajaanza kuonyesha dalili na ishara za ugonjwa huo.
-•  Toa taarifa haraka kwa wahudumu wa afya ya jamii (CHV) ndapo kuna mkaazi au  mmepokea mgeni  ana dalili za Korona
-•  Ugonjwa wa Korona kwa sasa hauna tiba wala chanjo na unaenea kwa kasi duniani. 
-•  Una wajibu wa kujikinga na kuwakinga wengine
-•  Unapohisi dalili au ishara za ugonjwa wa mafua makali baki nyumbani na piga simu kwa kutumia namba. Piga bila gharama 190
-•  Pia naweza kuwaunga kwenye Facebook,insta na whats app za kitengo cha elimu ya kinga wizara ya afya ili muweze pata taarifa za ukweli zaidi na mwenendo na matukio ya Korona Zanzibar
-</t>
-  </si>
-  <si>
-    <t>mask_questions</t>
-  </si>
-  <si>
-    <t>Questions about the mask</t>
-  </si>
-  <si>
-    <t>Masuali kuhusu barakoa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select_one yes_no </t>
-  </si>
-  <si>
-    <t>has_mask</t>
-  </si>
-  <si>
-    <t>Do you have a face mask (even a home made face mask) to cover mouth and face when exiting your home?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unayo Barakoa ( Hata ile ya kutengeneza nyumbani) kwa ajili ya kufunika mdomo na uso kila mara  unapotoka nyumbani kwako? </t>
-  </si>
-  <si>
-    <t>is_wearing</t>
-  </si>
-  <si>
-    <t>Are you wearing your mask every time you leave home?</t>
-  </si>
-  <si>
-    <t>Je umevaa barako yako  Kila muda unapotoka nyumbani?</t>
-  </si>
-  <si>
-    <t>selected(${has_mask},"yes")</t>
-  </si>
-  <si>
-    <t>not_wearing_msg</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Please direct how to prepare your mask at home by following the steps:&lt;/.span&gt;</t>
-  </si>
-  <si>
-    <t>&lt;span style="color:#f58a1f"&gt;Tafadhali muelekeze Jinsi anaweza kutengeneza barako yako nyumbani kwa kufuata hatua zifuatazo: &lt;/span&gt;</t>
-  </si>
-  <si>
-    <t>selected(${is_wearing},"no")</t>
-  </si>
-  <si>
-    <t>self_made_mask_pics</t>
-  </si>
-  <si>
-    <t>This is how you can make your cloth mask at home</t>
-  </si>
-  <si>
-    <t>Jinsi ya kutengeneza barakoa yako nyumbani.</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fold bandana in half </t>
-  </si>
-  <si>
-    <t>Kunja leso/kitambaa kiwe nusu</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic1.png</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fold top down, fold bottom up </t>
-  </si>
-  <si>
-    <t>Kunja sehemu ya juu kwa chini, na sehemu ya chini kwa juu</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic2.png</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Place the rubber bands or hair tiers about 6 inches apart </t>
-  </si>
-  <si>
-    <t>Weka mpira au vibanio vya nywelekila upande kwa kuacha nafasi ya inchi 6 katikati</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic3.png</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fold side to the middle and tuck </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kunja sehemu za mwisho/pembeni kuelekea katikati halafu shona/uibane  </t>
-  </si>
-  <si>
-    <t>self_made_mask_pic4.png</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic5</t>
-  </si>
-  <si>
-    <t>Mask as seen after preparing</t>
-  </si>
-  <si>
-    <t>Muonekano wa barakoa baada ya kuiandaa</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic5.png</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mask as seen after wearing </t>
-  </si>
-  <si>
-    <t>Muonekano wa barakoa baada ya kuvaa</t>
-  </si>
-  <si>
-    <t>self_made_mask_pic6.png</t>
-  </si>
-  <si>
-    <t>mask_importance</t>
-  </si>
-  <si>
-    <t>Remember that it is important to wear the mask to make sure they do not spread the virus to others. It is possible to spread the virus to others even if they have no symptoms at all.
-Wearing this mask will not protect you from getting sick if someone around you is sick, so it is important to maintain distance from other people and wash your hands often.Be careful and do not touch the outside or inside with your hands. Wash your hands with water and soap immediately before putting the mask on, and after taking it off. Wash your mask with soap and water daily after use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kumbuka ni muhimu sana kuvaa barakoa kila mara unapotoka nyumbani ili kuwalinda wengine, inawezekana kabisa kuwa na ugonjwa huu na kutoonesha dalili yeyote.
-Kuvaa barakoa hakukuepushi na kupata ugonjwa endapo utakua karibu sana na mgonjwa, hivyo basi ni muhimu kuendelea kukaa umbali kutoka kwa watu wengine na kuosha mikono yako kila mara.
-Kuwa makini na kushika barakoa yako kwa ndani au nje kwa mikono. Kosha mikono yako kwa maji na sabauni mara baada ya kuvaa au kuvua barakoa, Kosha barakoa yako kwa maji na sabuni kila siku baada ya kutumia.
-</t>
-  </si>
-  <si>
-    <t>Questions about hand washing</t>
-  </si>
-  <si>
-    <t>Maswali kuhusu uoshaji wa mikono</t>
-  </si>
-  <si>
-    <t>has_infrastructure</t>
-  </si>
-  <si>
-    <t>Are there any good infrastructures on handwashing at home?</t>
-  </si>
-  <si>
-    <t>Je nyumbani kuna miundombinu mizuri kwa ajili ya kuosha mikono kwa maji tiririka?</t>
-  </si>
-  <si>
-    <t>select_one is_practicing</t>
-  </si>
-  <si>
-    <t>is_practicing</t>
-  </si>
-  <si>
-    <t>How many times do you practice handwashing at home?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je ni mara ngapi unaosha mikono kwa maji tiririka na sabuni ukiwa nyumbani? </t>
-  </si>
-  <si>
-    <t>practice_reminder</t>
-  </si>
-  <si>
-    <t>Its important to practice hand washing every time you go outside the house to make sure you protectect yourself and other people from Corona virus.</t>
-  </si>
-  <si>
-    <t>Ni muhimu kuosha mikono kwa maji tiririka na sabuni mara kwa mara  ili kujilinda na kuwalinda wengine kutokana na ugojwa wa korona.</t>
-  </si>
-  <si>
-    <t>risks_and_directions</t>
-  </si>
-  <si>
-    <t>Questions about risks and directions to household members</t>
-  </si>
-  <si>
-    <t>Maswali kuhusu makundi hatarishi na maelekezo kwa wanakaya</t>
-  </si>
-  <si>
-    <t>select_multiple serious_diseases</t>
-  </si>
-  <si>
     <t>serious_diseases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is anyone in your household suffering from these serious diseases? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je kuna yeyote kwenye kaya yenu anasumbuliwa na magonjwa haya hatarishi? </t>
-  </si>
-  <si>
-    <t>(selected(.,"none") and count-selected(.)=1) or (not(selected(.,"none")) and count-selected(.)&gt;=1)</t>
-  </si>
-  <si>
-    <t>Cannot select "None of the above" and another option.</t>
-  </si>
-  <si>
-    <t>Huwezi kuchaguwa "Hakuna mojawapo" na chaguo jengine</t>
-  </si>
-  <si>
-    <t>age_above_50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is someone in your household older than 50? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je kwenye kaya yenu kuna mtu mwenye umri Zaidi ya miaka 50? </t>
-  </si>
-  <si>
-    <t>prevention_for_elderly</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Older people and any aged people with health problems like the one I mentioned above are more at risk of getting coronavirus disease. Be more careful with them, We strongly recommend they stay home and avoid any gatherings and when they experience any symptoms please call the emergency help line as soon as possible to save their lives.</t>
-  </si>
-  <si>
-    <t>Watu  wazima na wale wenye umri mkubwa na wenye matatizo ya kiafya kama niliyotaja hapo juu wapo katika hatari zaidi ya kupata  maradhi ya korona, tuwe makini nao zaidi, Tunashauri wabaki nyumbani na waepuke mikusanyiko ya aina yeyote,na wanapopata dalili zozote tafadhali piga namba ya msaada wa dharura haraka iwezekanavyo kunusuru maisha yao.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_understading </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Questions to test understanding</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Maswali ya kupima uelewa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">asymptomatic </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you think people who do not show any signs of illness such as coughing or sneezing can spread the virus / spread the disease? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Je unadhani watu wasioonesha dalili zozote za ugonjwa kama vile kukohoa au kupiga chafya  wanaweza kusambaza virusi/kueneza ugonjwa? </t>
-  </si>
-  <si>
-    <t>infected_area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is it possible for a person to get infected by touching the infected area? </t>
-  </si>
-  <si>
-    <t>Je inawezekana kwa mtu kupata virusi/kuambukizwa kwa kugusa sehemu yenye virusi ?</t>
-  </si>
-  <si>
-    <t>educate_client</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The answer to both questions is Yes. People who show no signs of illness can spread the disease. It is possible for a person to get infected by touching an infected area and then touching their face. This is why it is important to always wear a mask outside of the home, and wash hands frequently with soap.
-Thank you for your attention
-</t>
-  </si>
-  <si>
-    <t>Majibu ya maswali yote mawili ni Ndio.Watu wasioonesha dalili wanaweza kueneza maambukizi. Inawezekana kwa mtu kuathirika kwa kushika sehemu yenye virusi na baadae kushika uso wake. Kwahiyo ni muhimu kuvaa barakoa muda wote unapotoka nyumbani , kuosha mikono mara kwa mara  kwa maji na sabuni.Ahsanteni kwa kunisikilia na kwa ushirikiano wenu.</t>
   </si>
   <si>
     <t>list_name</t>
@@ -993,15 +401,261 @@
   <si>
     <t>data</t>
   </si>
+  <si>
+    <t>corona_precautions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precautions against Corona </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tahadhari juu ya Korona </t>
+  </si>
+  <si>
+    <t>does_client_take_precautions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je bado unachukua tahadhari juu ya ugonjwa wa Korona? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are you still taking precautions against COVID ? </t>
+  </si>
+  <si>
+    <t>select_multiple precations_taken</t>
+  </si>
+  <si>
+    <t>precautions_taken</t>
+  </si>
+  <si>
+    <t>Muombe mlengwa akutajie tahadhari hizo, muhudumu (CHV) jaza kwenye kila alioitaja hapo chini.</t>
+  </si>
+  <si>
+    <t>selected(${does_client_take_precautions},"yes")</t>
+  </si>
+  <si>
+    <t>precations_taken</t>
+  </si>
+  <si>
+    <t>Nawa mikono kwa  maji safi ya kutiririka na sabuni mara kwa mara(angalau kwa sekunde 20)</t>
+  </si>
+  <si>
+    <t>Epuka kukaa kwenye mikusanyiko ya watu na ukae umbali wa mita moja</t>
+  </si>
+  <si>
+    <t>Funika mdomo na pua kwa kitambaa, tishu au kiwiko cha mkono unapopiga chafya, kukohoa au kupenga mafua.</t>
+  </si>
+  <si>
+    <t>Epuka tabia ya  kupeana mikono</t>
+  </si>
+  <si>
+    <t>Epuka kushika  mdomo, pua na macho kabla ya kuosha mikono</t>
+  </si>
+  <si>
+    <t>Epuka safari zisizo za lazima</t>
+  </si>
+  <si>
+    <t>Kumbuka kuosha mikono kwa sababuni na maji tiririka muda wote kabla ya kuingia nyumbani</t>
+  </si>
+  <si>
+    <t>Kumbuka Kuvaa barakoa muda wote unapotoka nje ya nyumba yako.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nyengine</t>
+  </si>
+  <si>
+    <t>avoid_gathering</t>
+  </si>
+  <si>
+    <t>cover_mouth</t>
+  </si>
+  <si>
+    <t>avoid_handshake</t>
+  </si>
+  <si>
+    <t>avoid_face_touch</t>
+  </si>
+  <si>
+    <t>avoid_unnecessary_travel</t>
+  </si>
+  <si>
+    <t>regular_hand_wash</t>
+  </si>
+  <si>
+    <t>hand_wash_before_home</t>
+  </si>
+  <si>
+    <t>wear_mask</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">congratulate_client </t>
+  </si>
+  <si>
+    <t>Mpongeze mama/mlezi, vizuri, ni vyema kuendelea kuchukua tahadhari juu ya Ugonjwa wa Corona, pia amjuilishe mlengwa ugonjwa huo bado upo na unaendelea kuathiri nchi nyingi ikiwemo nchi yetu na nchi jirani.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selected(${precautions_taken},"regular_hand_wash") or selected(${precautions_taken},"avoid_gathering") or selected(${precautions_taken},"cover_mouth") or selected(${precautions_taken},"avoid_handshake") or selected(${precautions_taken},"avoid_face_touch") or selected(${precautions_taken},"avoid_unnecessary_travel") or selected(${precautions_taken},"hand_wash_before_home") or selected(${precautions_taken},"wear_mask") or selected(${precautions_taken},"other") </t>
+  </si>
+  <si>
+    <t>read_precautions_to_client</t>
+  </si>
+  <si>
+    <t>&lt;span style="color:#f58a1f"&gt;Msomee mama/mlezi tahadhari hizi.&lt;/span&gt;
+•	Nawa mikono kwa  maji safi ya kutiririka na sabuni mara kwa mara(angalau kwa sekunde 20) (Wafundishe kutengeneza kibuyu chirizi kama hamna mferji)
+•	Epuka kukaa kwenye mikusanyiko ya watu na ukae umbali wa mita moja 
+•	Funika mdomo na pua kwa kitambaa, tishu au kiwiko cha mkono unapopiga chafya, kukohoa au kupenga mafua
+•	Epuka tabia ya  kupeana mikono
+•	Epuka kushika  mdomo, pua na macho kabla ya kuosha mikono
+•	Epuka safari zisizo za lazima
+•	Kumbuka kuosha mikono kwa sababuni na maji tiririka muda wote kabla ya kuingia nyumbani
+•	Kumbuka Kuvaa barakoa muda wote unapotoka nje ya nyumba yako.</t>
+  </si>
+  <si>
+    <t>selected(${does_client_take_precautions},"no")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">corona_signs </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signs of Corona </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dailili za Korona </t>
+  </si>
+  <si>
+    <t>corona_signs_list</t>
+  </si>
+  <si>
+    <t>Baadhi ya dalili na ishara za ugonjwa wa korona, kwa maelezo zaidi ya dalili za ugonjwa huu tuwasiliane na madaktari wa vituo vya afya maana dalili hizo hubadilika mara kawa mara.
+• Kupata homa kali 
+• Kukohoa 
+• Kupumua kwa shida
+• Chafya za mara kwa mara 
+• Kupata mafua makali 
+• Kuumwa na kichwa 
+• Vidonda vya koo na 
+• Kutohisi ladha ya chakula au kutosikia harufu
+• Kuumwa na viungo vya mwili.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je kwenye kaya yenu kuna mtu mwenye umri zaidi ya miaka 50? </t>
+  </si>
+  <si>
+    <t>corona_education</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corona Education </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elimu juu ya Korona </t>
+  </si>
+  <si>
+    <t>source_of_corona_education</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_multiple source_of_corona_education </t>
+  </si>
+  <si>
+    <t>media_outlet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vyombo vya Habari </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media Outlets </t>
+  </si>
+  <si>
+    <t>billboards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill boards </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mabango barabarani </t>
+  </si>
+  <si>
+    <t>social_media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Social Media </t>
+  </si>
+  <si>
+    <t>Mitandao ya kijamii</t>
+  </si>
+  <si>
+    <t>Nyengine</t>
+  </si>
+  <si>
+    <t>Vipeperushi</t>
+  </si>
+  <si>
+    <t>flyers</t>
+  </si>
+  <si>
+    <t>source_of_corona_education_other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please specify </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tafadhali taja </t>
+  </si>
+  <si>
+    <t>selected(${source_of_corona_education},"other")</t>
+  </si>
+  <si>
+    <t>vulnerable_corona_group</t>
+  </si>
+  <si>
+    <t>Makundi hatarishi na watu walio hatarini kupata maradhi ya korona.</t>
+  </si>
+  <si>
+    <t>list_of_vulnerable_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Watu wazima na wale wenye umri mkubwa na wenye matatizo ya kiafya kama vile
+• Magonjwa ya moyo
+• Kisukari
+• Magonjwa sugu ya kupumua
+• Saratani
+• Shinikizo la damu/presha
+• Pumu
+• Ugonjwa wa figo/ugonjwa waini
+ Wapo katika hatari zaidi ya kupata  maradhi ya korona, tuwe makini nao zaidi, Tunashauri wabaki nyumbani na waepuke mikusanyiko ya aina yeyote,na wanapopata dalili zozote waende kituo cha afya au kupiga namba ya msaada wa dharura haraka iwezekanavyo kunusuru maisha yao.</t>
+  </si>
+  <si>
+    <t>corona_signs</t>
+  </si>
+  <si>
+    <t>Je, ni wapi unapata zaidi elimu kuhusu Korona?</t>
+  </si>
+  <si>
+    <t>age_above_50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;As a CHV you should avoid spreading corona virus, therefore take below precautions while conducting visits.
+•	Conduct visits in a ventilated area, keep the distance of two meters from a client, wear mask all the time, and avoid hands shaking with a client during conducting visits.
+•	Wash your hands frequently with clean water and soap or sanitize your hands, avoid crowds and cover your mouth while sneezing or coughing.
+•	Do not go for a visit if you have symptoms of fever, cough or frequent sneezing.&lt;/span&gt; 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;span style="color:#f58a1f"&gt;Kama muhudumu wa afya kwenye jamii, epuka kusambaza maambukizi ya ugonjwa wa korona, hivyo zingatia yafuatayo wakati wa kutuo huduma.
+• Kaa mahali palipo na  mzunguko mzuri wa hewa, umbali wa mita mbili, ukiwa umevaa barakoa, pasipo kushikana mikoni na mteja wako wakati wote wa kufanya matembeleo.
+• Osha mikono yako kwa sabuni au kitakasa mikono mara kwa mara wakati wa kufanya tembeleo, epuka mikusanyiko,funika mdomo wako kwa kitambaa au kiwiko unavyooenda chafya au kukohoa,
+• Tafadhali usiende kutoa huduma ukijihisi na dalili za homa na kukohoa na kwenda chafya kwa wingi.&lt;/span&gt; 
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1011,15 +665,18 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1035,6 +692,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1045,10 +703,30 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1111,7 +789,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1128,7 +806,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1149,6 +826,20 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1363,15 +1054,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1033"/>
+  <dimension ref="A1:Z1035"/>
   <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="23.54296875" customWidth="1"/>
-    <col min="3" max="3" width="286.6796875" customWidth="1"/>
+    <col min="3" max="3" width="55.453125" customWidth="1"/>
     <col min="4" max="26" width="23.54296875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1997,11 +1688,11 @@
       <c r="B18" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>51</v>
+      <c r="C18" s="39" t="s">
+        <v>195</v>
       </c>
-      <c r="D18" s="15" t="s">
-        <v>52</v>
+      <c r="D18" s="39" t="s">
+        <v>196</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -2028,7 +1719,7 @@
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1">
       <c r="A19" s="12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>45</v>
@@ -2059,21 +1750,21 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>19</v>
+      <c r="A20" s="27" t="s">
+        <v>44</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>54</v>
+      <c r="B20" s="27" t="s">
+        <v>126</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>55</v>
+      <c r="C20" s="31" t="s">
+        <v>127</v>
       </c>
-      <c r="D20" s="16" t="s">
-        <v>56</v>
+      <c r="D20" s="31" t="s">
+        <v>128</v>
       </c>
-      <c r="E20" s="16"/>
-      <c r="G20" s="2" t="s">
-        <v>57</v>
+      <c r="E20" s="15"/>
+      <c r="G20" s="33" t="s">
+        <v>52</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -2096,23 +1787,25 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A21" s="16" t="s">
-        <v>49</v>
+      <c r="A21" s="27" t="s">
+        <v>53</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>58</v>
+      <c r="B21" s="27" t="s">
+        <v>129</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>59</v>
+      <c r="C21" s="27" t="s">
+        <v>131</v>
       </c>
-      <c r="D21" s="16" t="s">
-        <v>60</v>
+      <c r="D21" s="31" t="s">
+        <v>130</v>
       </c>
-      <c r="E21" s="2"/>
+      <c r="E21" s="31" t="s">
+        <v>54</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
-      <c r="I21" s="17"/>
+      <c r="I21" s="16"/>
       <c r="J21" s="1"/>
       <c r="K21" s="8"/>
       <c r="L21" s="1"/>
@@ -2132,25 +1825,25 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="14.75">
-      <c r="A22" s="16" t="s">
-        <v>61</v>
+      <c r="A22" s="27" t="s">
+        <v>132</v>
       </c>
-      <c r="B22" s="16" t="s">
-        <v>62</v>
+      <c r="B22" s="27" t="s">
+        <v>133</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>63</v>
+      <c r="C22" s="15"/>
+      <c r="D22" s="17" t="s">
+        <v>134</v>
       </c>
-      <c r="D22" s="18" t="s">
-        <v>64</v>
+      <c r="E22" s="31" t="s">
+        <v>54</v>
       </c>
-      <c r="E22" s="16" t="s">
-        <v>65</v>
+      <c r="F22" s="1" t="s">
+        <v>135</v>
       </c>
-      <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="17"/>
+      <c r="I22" s="16"/>
       <c r="J22" s="1"/>
       <c r="K22" s="8"/>
       <c r="L22" s="1"/>
@@ -2170,25 +1863,23 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" spans="1:26" ht="13">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>66</v>
+      <c r="B23" s="34" t="s">
+        <v>155</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>68</v>
+      <c r="C23" s="15"/>
+      <c r="D23" s="33" t="s">
+        <v>156</v>
       </c>
       <c r="E23" s="2"/>
-      <c r="F23" s="19" t="s">
-        <v>69</v>
+      <c r="F23" s="34" t="s">
+        <v>157</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="17"/>
+      <c r="I23" s="16"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
@@ -2207,64 +1898,56 @@
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" spans="1:26" ht="13">
-      <c r="A24" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="1"/>
-      <c r="W24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="1"/>
-      <c r="Z24" s="1"/>
-    </row>
-    <row r="25" spans="1:26" ht="13">
-      <c r="A25" s="16" t="s">
+    <row r="24" spans="1:26" s="31" customFormat="1" ht="59.5" customHeight="1">
+      <c r="A24" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="16" t="s">
-        <v>73</v>
+      <c r="B24" s="34" t="s">
+        <v>158</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>74</v>
+      <c r="C24" s="30"/>
+      <c r="D24" s="35" t="s">
+        <v>159</v>
       </c>
-      <c r="D25" s="16" t="s">
-        <v>75</v>
+      <c r="E24" s="30"/>
+      <c r="F24" s="34" t="s">
+        <v>160</v>
       </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="19" t="s">
-        <v>76</v>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
+      <c r="V24" s="27"/>
+      <c r="W24" s="27"/>
+      <c r="X24" s="27"/>
+      <c r="Y24" s="27"/>
+      <c r="Z24" s="27"/>
+    </row>
+    <row r="25" spans="1:26" ht="13">
+      <c r="A25" s="31" t="s">
+        <v>51</v>
       </c>
+      <c r="B25" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+      <c r="I25" s="2"/>
       <c r="J25" s="1"/>
       <c r="K25" s="8"/>
       <c r="L25" s="1"/>
@@ -2284,211 +1967,199 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="13">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+    </row>
+    <row r="27" spans="1:26" ht="260">
+      <c r="A27" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="21" t="s">
-        <v>77</v>
+      <c r="B27" s="34" t="s">
+        <v>164</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>78</v>
+      <c r="C27" s="20"/>
+      <c r="D27" s="36" t="s">
+        <v>165</v>
       </c>
-      <c r="D26" s="21" t="s">
-        <v>79</v>
+      <c r="E27" s="19"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="3"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+      <c r="X27" s="3"/>
+      <c r="Y27" s="3"/>
+      <c r="Z27" s="3"/>
+    </row>
+    <row r="28" spans="1:26" ht="13">
+      <c r="A28" s="34" t="s">
+        <v>53</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="22" t="s">
-        <v>76</v>
+      <c r="B28" s="27" t="s">
+        <v>194</v>
       </c>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
-      <c r="S26" s="3"/>
-      <c r="T26" s="3"/>
-      <c r="U26" s="3"/>
-      <c r="V26" s="3"/>
-      <c r="W26" s="3"/>
-      <c r="X26" s="3"/>
-      <c r="Y26" s="3"/>
-      <c r="Z26" s="3"/>
-    </row>
-    <row r="27" spans="1:26" ht="13">
-      <c r="A27" s="16" t="s">
-        <v>80</v>
+      <c r="C28" s="15"/>
+      <c r="D28" s="33" t="s">
+        <v>166</v>
       </c>
-      <c r="B27" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F27" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1"/>
-      <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="1"/>
-      <c r="U27" s="1"/>
-      <c r="V27" s="1"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-    </row>
-    <row r="28" spans="1:26" ht="13">
-      <c r="A28" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
-      <c r="S28" s="3"/>
-      <c r="T28" s="3"/>
-      <c r="U28" s="3"/>
-      <c r="V28" s="3"/>
-      <c r="W28" s="3"/>
-      <c r="X28" s="3"/>
-      <c r="Y28" s="3"/>
-      <c r="Z28" s="3"/>
-    </row>
-    <row r="29" spans="1:26" ht="13">
-      <c r="A29" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B29" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F29" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
-      <c r="V29" s="1"/>
-      <c r="W29" s="1"/>
-      <c r="X29" s="1"/>
-      <c r="Y29" s="1"/>
-      <c r="Z29" s="1"/>
-    </row>
-    <row r="30" spans="1:26" ht="13">
-      <c r="A30" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="16" t="s">
+      <c r="E28" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="1"/>
-      <c r="W30" s="1"/>
-      <c r="X30" s="1"/>
-      <c r="Y30" s="1"/>
-      <c r="Z30" s="1"/>
-    </row>
-    <row r="31" spans="1:26" ht="13">
-      <c r="A31" s="16" t="s">
+      <c r="F28" s="21"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1"/>
+    </row>
+    <row r="29" spans="1:26" s="31" customFormat="1" ht="13">
+      <c r="A29" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>192</v>
+      </c>
+      <c r="C29" s="30"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
+      <c r="V29" s="27"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+    </row>
+    <row r="30" spans="1:26" ht="13">
+      <c r="A30" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="16" t="s">
-        <v>91</v>
+      <c r="B30" s="34" t="s">
+        <v>167</v>
       </c>
-      <c r="C31" s="16" t="s">
-        <v>92</v>
+      <c r="C30" s="34" t="s">
+        <v>168</v>
       </c>
-      <c r="D31" s="16" t="s">
-        <v>93</v>
+      <c r="D30" s="34" t="s">
+        <v>169</v>
       </c>
-      <c r="E31" s="2"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="19" t="s">
+      <c r="E30" s="19"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="34" t="s">
         <v>48</v>
       </c>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+      <c r="V30" s="3"/>
+      <c r="W30" s="3"/>
+      <c r="X30" s="3"/>
+      <c r="Y30" s="3"/>
+      <c r="Z30" s="3"/>
+    </row>
+    <row r="31" spans="1:26" ht="13">
+      <c r="A31" s="34" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="C31" s="15"/>
+      <c r="D31" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="E31" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="F31" s="21"/>
+      <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
@@ -2509,26 +2180,30 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" spans="1:26" ht="14.25">
-      <c r="A32" s="16" t="s">
-        <v>49</v>
+    <row r="32" spans="1:26" ht="13">
+      <c r="A32" s="34" t="s">
+        <v>56</v>
       </c>
-      <c r="B32" s="16" t="s">
-        <v>94</v>
+      <c r="B32" s="34" t="s">
+        <v>184</v>
       </c>
-      <c r="C32" s="24" t="s">
-        <v>95</v>
+      <c r="C32" s="33" t="s">
+        <v>185</v>
       </c>
-      <c r="D32" s="16" t="s">
-        <v>96</v>
+      <c r="D32" s="33" t="s">
+        <v>186</v>
       </c>
-      <c r="E32" s="2"/>
-      <c r="F32" s="1"/>
+      <c r="E32" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="F32" s="34" t="s">
+        <v>187</v>
+      </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="8"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
@@ -2546,21 +2221,21 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="13">
-      <c r="A33" s="16" t="s">
-        <v>53</v>
+      <c r="A33" s="34" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="16" t="s">
-        <v>91</v>
+      <c r="B33" s="34" t="s">
+        <v>167</v>
       </c>
-      <c r="C33" s="31"/>
-      <c r="D33" s="32"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
       <c r="E33" s="2"/>
       <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
+      <c r="G33" s="18"/>
       <c r="H33" s="1"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="8"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
@@ -2577,28 +2252,26 @@
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
     </row>
-    <row r="34" spans="1:26" ht="13">
-      <c r="A34" s="16" t="s">
-        <v>19</v>
+    <row r="34" spans="1:26" ht="14.25">
+      <c r="A34" s="34" t="s">
+        <v>44</v>
       </c>
-      <c r="B34" s="16" t="s">
-        <v>97</v>
+      <c r="B34" s="34" t="s">
+        <v>188</v>
       </c>
-      <c r="C34" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="D34" s="16" t="s">
-        <v>99</v>
+      <c r="C34" s="23"/>
+      <c r="D34" s="33" t="s">
+        <v>189</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="1"/>
-      <c r="G34" s="19" t="s">
+      <c r="G34" s="34" t="s">
         <v>48</v>
       </c>
       <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="8"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
@@ -2615,26 +2288,24 @@
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
     </row>
-    <row r="35" spans="1:26" ht="13">
-      <c r="A35" s="16" t="s">
+    <row r="35" spans="1:26" ht="72" customHeight="1">
+      <c r="A35" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B35" s="16" t="s">
-        <v>100</v>
+      <c r="B35" s="34" t="s">
+        <v>190</v>
       </c>
-      <c r="C35" s="16" t="s">
-        <v>101</v>
+      <c r="C35" s="30"/>
+      <c r="D35" s="35" t="s">
+        <v>191</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="E35" s="2"/>
+      <c r="E35" s="35"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="8"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
@@ -2652,20 +2323,21 @@
       <c r="Z35" s="1"/>
     </row>
     <row r="36" spans="1:26" ht="13">
-      <c r="A36" s="16" t="s">
-        <v>29</v>
+      <c r="A36" s="34" t="s">
+        <v>51</v>
       </c>
-      <c r="B36" s="16" t="s">
-        <v>97</v>
+      <c r="B36" s="34" t="s">
+        <v>188</v>
       </c>
-      <c r="C36" s="16"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
       <c r="E36" s="2"/>
       <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
+      <c r="G36" s="18"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
-      <c r="K36" s="1"/>
+      <c r="K36" s="8"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
@@ -2683,27 +2355,17 @@
       <c r="Z36" s="1"/>
     </row>
     <row r="37" spans="1:26" ht="13">
-      <c r="A37" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B37" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="C37" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="D37" s="16" t="s">
-        <v>105</v>
-      </c>
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
       <c r="E37" s="2"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
+      <c r="K37" s="8"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
@@ -2721,25 +2383,16 @@
       <c r="Z37" s="1"/>
     </row>
     <row r="38" spans="1:26" ht="13">
-      <c r="A38" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="D38" s="16" t="s">
-        <v>108</v>
-      </c>
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
       <c r="E38" s="2"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
-      <c r="K38" s="8"/>
+      <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
@@ -2757,27 +2410,17 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="13">
-      <c r="A39" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>65</v>
-      </c>
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="2"/>
       <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
+      <c r="G39" s="18"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
-      <c r="K39" s="8"/>
+      <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
@@ -2795,22 +2438,12 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="13">
-      <c r="A40" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>114</v>
-      </c>
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
       <c r="E40" s="2"/>
-      <c r="F40" s="19" t="s">
-        <v>115</v>
-      </c>
+      <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -2833,33 +2466,25 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="13">
-      <c r="A41" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="C41" s="31"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="1"/>
+      <c r="A41" s="15"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
+      <c r="K41" s="8"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
       <c r="Q41" s="1"/>
-      <c r="R41" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="S41" s="16" t="s">
-        <v>117</v>
-      </c>
+      <c r="R41" s="1"/>
+      <c r="S41" s="1"/>
       <c r="T41" s="1"/>
       <c r="U41" s="1"/>
       <c r="V41" s="1"/>
@@ -2869,33 +2494,25 @@
       <c r="Z41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="13">
-      <c r="A42" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="18"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
+      <c r="K42" s="8"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
-      <c r="R42" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="S42" s="19" t="s">
-        <v>119</v>
-      </c>
+      <c r="R42" s="1"/>
+      <c r="S42" s="1"/>
       <c r="T42" s="1"/>
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
@@ -2905,14 +2522,10 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="13">
-      <c r="A43" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="38"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -2926,12 +2539,8 @@
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
-      <c r="R43" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="S43" s="19" t="s">
-        <v>121</v>
-      </c>
+      <c r="R43" s="15"/>
+      <c r="S43" s="15"/>
       <c r="T43" s="1"/>
       <c r="U43" s="1"/>
       <c r="V43" s="1"/>
@@ -2941,12 +2550,8 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="13">
-      <c r="A44" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B44" s="19" t="s">
-        <v>103</v>
-      </c>
+      <c r="A44" s="18"/>
+      <c r="B44" s="15"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -2962,8 +2567,8 @@
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
-      <c r="R44" s="1"/>
-      <c r="S44" s="1"/>
+      <c r="R44" s="18"/>
+      <c r="S44" s="18"/>
       <c r="T44" s="1"/>
       <c r="U44" s="1"/>
       <c r="V44" s="1"/>
@@ -2973,23 +2578,13 @@
       <c r="Z44" s="1"/>
     </row>
     <row r="45" spans="1:26" ht="13">
-      <c r="A45" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" s="19" t="s">
-        <v>122</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="D45" s="19" t="s">
-        <v>124</v>
-      </c>
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-      <c r="G45" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
@@ -3000,8 +2595,8 @@
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
-      <c r="R45" s="1"/>
-      <c r="S45" s="1"/>
+      <c r="R45" s="18"/>
+      <c r="S45" s="18"/>
       <c r="T45" s="1"/>
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
@@ -3011,18 +2606,10 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="13">
-      <c r="A46" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="19" t="s">
-        <v>125</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="D46" s="19" t="s">
-        <v>127</v>
-      </c>
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
@@ -3047,17 +2634,13 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="13">
-      <c r="A47" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B47" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
+      <c r="G47" s="18"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
@@ -3068,12 +2651,8 @@
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
-      <c r="R47" s="19" t="s">
-        <v>129</v>
-      </c>
-      <c r="S47" s="19" t="s">
-        <v>129</v>
-      </c>
+      <c r="R47" s="1"/>
+      <c r="S47" s="1"/>
       <c r="T47" s="1"/>
       <c r="U47" s="1"/>
       <c r="V47" s="1"/>
@@ -3083,14 +2662,10 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="13">
-      <c r="A48" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
@@ -3104,12 +2679,8 @@
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
-      <c r="R48" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="S48" s="19" t="s">
-        <v>131</v>
-      </c>
+      <c r="R48" s="1"/>
+      <c r="S48" s="1"/>
       <c r="T48" s="1"/>
       <c r="U48" s="1"/>
       <c r="V48" s="1"/>
@@ -3119,14 +2690,10 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="13">
-      <c r="A49" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
+      <c r="A49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
@@ -3140,12 +2707,8 @@
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
-      <c r="R49" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="S49" s="19" t="s">
-        <v>133</v>
-      </c>
+      <c r="R49" s="18"/>
+      <c r="S49" s="18"/>
       <c r="T49" s="1"/>
       <c r="U49" s="1"/>
       <c r="V49" s="1"/>
@@ -3155,14 +2718,10 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="13">
-      <c r="A50" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
+      <c r="A50" s="18"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
@@ -3176,12 +2735,8 @@
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
-      <c r="R50" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="S50" s="19" t="s">
-        <v>135</v>
-      </c>
+      <c r="R50" s="18"/>
+      <c r="S50" s="18"/>
       <c r="T50" s="1"/>
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
@@ -3191,14 +2746,10 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" spans="1:26" ht="13">
-      <c r="A51" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="C51" s="19"/>
-      <c r="D51" s="19"/>
+      <c r="A51" s="18"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
@@ -3212,12 +2763,8 @@
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
-      <c r="R51" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="S51" s="19" t="s">
-        <v>137</v>
-      </c>
+      <c r="R51" s="18"/>
+      <c r="S51" s="18"/>
       <c r="T51" s="1"/>
       <c r="U51" s="1"/>
       <c r="V51" s="1"/>
@@ -3227,14 +2774,10 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="13">
-      <c r="A52" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="C52" s="19"/>
-      <c r="D52" s="19"/>
+      <c r="A52" s="18"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
@@ -3248,12 +2791,8 @@
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
-      <c r="R52" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="S52" s="19" t="s">
-        <v>139</v>
-      </c>
+      <c r="R52" s="18"/>
+      <c r="S52" s="18"/>
       <c r="T52" s="1"/>
       <c r="U52" s="1"/>
       <c r="V52" s="1"/>
@@ -3263,14 +2802,10 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="13">
-      <c r="A53" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
+      <c r="A53" s="18"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
@@ -3284,8 +2819,8 @@
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
-      <c r="R53" s="1"/>
-      <c r="S53" s="1"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
       <c r="T53" s="1"/>
       <c r="U53" s="1"/>
       <c r="V53" s="1"/>
@@ -3295,22 +2830,13 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" spans="1:26" ht="13">
-      <c r="A54" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B54" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>143</v>
-      </c>
+      <c r="A54" s="18"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
       <c r="E54" s="1"/>
-      <c r="G54" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
@@ -3321,8 +2847,8 @@
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
-      <c r="R54" s="1"/>
-      <c r="S54" s="1"/>
+      <c r="R54" s="18"/>
+      <c r="S54" s="18"/>
       <c r="T54" s="1"/>
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
@@ -3332,18 +2858,10 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="13">
-      <c r="A55" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B55" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="D55" s="19" t="s">
-        <v>146</v>
-      </c>
+      <c r="A55" s="18"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
@@ -3368,17 +2886,12 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="13">
-      <c r="A56" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B56" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
+      <c r="A56" s="18"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
       <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
+      <c r="G56" s="18"/>
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
@@ -3400,23 +2913,13 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" spans="1:26" ht="13">
-      <c r="A57" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="C57" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="D57" s="19" t="s">
-        <v>149</v>
-      </c>
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
-      <c r="G57" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
@@ -3438,21 +2941,11 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="13">
-      <c r="A58" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="B58" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="D58" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="E58" s="19" t="s">
-        <v>65</v>
-      </c>
+      <c r="A58" s="18"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -3476,25 +2969,13 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="13">
-      <c r="A59" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B59" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="C59" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="D59" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="E59" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="F59" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="G59" s="1"/>
+      <c r="A59" s="18"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="18"/>
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
@@ -3516,22 +2997,12 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="13">
-      <c r="A60" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B60" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="D60" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="F60" s="19" t="s">
-        <v>161</v>
-      </c>
+      <c r="A60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="1"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
@@ -3554,20 +3025,12 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" spans="1:26" ht="13">
-      <c r="A61" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B61" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="C61" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="D61" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
@@ -3579,8 +3042,8 @@
       <c r="O61" s="1"/>
       <c r="P61" s="1"/>
       <c r="Q61" s="1"/>
-      <c r="R61" s="19"/>
-      <c r="S61" s="19"/>
+      <c r="R61" s="1"/>
+      <c r="S61" s="1"/>
       <c r="T61" s="1"/>
       <c r="U61" s="1"/>
       <c r="V61" s="1"/>
@@ -3590,20 +3053,12 @@
       <c r="Z61" s="1"/>
     </row>
     <row r="62" spans="1:26" ht="13">
-      <c r="A62" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B62" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="D62" s="19" t="s">
-        <v>167</v>
-      </c>
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
       <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
+      <c r="F62" s="18"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
@@ -3615,12 +3070,8 @@
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
-      <c r="R62" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="S62" s="19" t="s">
-        <v>168</v>
-      </c>
+      <c r="R62" s="1"/>
+      <c r="S62" s="1"/>
       <c r="T62" s="1"/>
       <c r="U62" s="1"/>
       <c r="V62" s="1"/>
@@ -3630,18 +3081,10 @@
       <c r="Z62" s="1"/>
     </row>
     <row r="63" spans="1:26" ht="13">
-      <c r="A63" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>169</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="D63" s="19" t="s">
-        <v>171</v>
-      </c>
+      <c r="A63" s="18"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
@@ -3655,12 +3098,8 @@
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
-      <c r="R63" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="S63" s="19" t="s">
-        <v>172</v>
-      </c>
+      <c r="R63" s="18"/>
+      <c r="S63" s="18"/>
       <c r="T63" s="1"/>
       <c r="U63" s="1"/>
       <c r="V63" s="1"/>
@@ -3670,18 +3109,10 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="13">
-      <c r="A64" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B64" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="D64" s="19" t="s">
-        <v>175</v>
-      </c>
+      <c r="A64" s="18"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
@@ -3695,12 +3126,8 @@
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
       <c r="Q64" s="1"/>
-      <c r="R64" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="S64" s="19" t="s">
-        <v>176</v>
-      </c>
+      <c r="R64" s="18"/>
+      <c r="S64" s="18"/>
       <c r="T64" s="1"/>
       <c r="U64" s="1"/>
       <c r="V64" s="1"/>
@@ -3710,18 +3137,10 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="13">
-      <c r="A65" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B65" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="C65" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="D65" s="19" t="s">
-        <v>179</v>
-      </c>
+      <c r="A65" s="18"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="18"/>
+      <c r="D65" s="18"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
@@ -3735,12 +3154,8 @@
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
       <c r="Q65" s="1"/>
-      <c r="R65" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="S65" s="19" t="s">
-        <v>180</v>
-      </c>
+      <c r="R65" s="18"/>
+      <c r="S65" s="18"/>
       <c r="T65" s="1"/>
       <c r="U65" s="1"/>
       <c r="V65" s="1"/>
@@ -3750,18 +3165,10 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="13">
-      <c r="A66" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B66" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="C66" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="D66" s="19" t="s">
-        <v>183</v>
-      </c>
+      <c r="A66" s="18"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
@@ -3775,12 +3182,8 @@
       <c r="O66" s="1"/>
       <c r="P66" s="1"/>
       <c r="Q66" s="1"/>
-      <c r="R66" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="S66" s="19" t="s">
-        <v>184</v>
-      </c>
+      <c r="R66" s="18"/>
+      <c r="S66" s="18"/>
       <c r="T66" s="1"/>
       <c r="U66" s="1"/>
       <c r="V66" s="1"/>
@@ -3790,18 +3193,10 @@
       <c r="Z66" s="1"/>
     </row>
     <row r="67" spans="1:26" ht="13">
-      <c r="A67" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B67" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="C67" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="D67" s="19" t="s">
-        <v>187</v>
-      </c>
+      <c r="A67" s="18"/>
+      <c r="B67" s="18"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="18"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
@@ -3815,12 +3210,8 @@
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
       <c r="Q67" s="1"/>
-      <c r="R67" s="19" t="s">
-        <v>188</v>
-      </c>
-      <c r="S67" s="19" t="s">
-        <v>188</v>
-      </c>
+      <c r="R67" s="18"/>
+      <c r="S67" s="18"/>
       <c r="T67" s="1"/>
       <c r="U67" s="1"/>
       <c r="V67" s="1"/>
@@ -3830,18 +3221,10 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="13">
-      <c r="A68" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B68" s="19" t="s">
-        <v>189</v>
-      </c>
-      <c r="C68" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="D68" s="19" t="s">
-        <v>191</v>
-      </c>
+      <c r="A68" s="18"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="18"/>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
@@ -3855,8 +3238,8 @@
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
       <c r="Q68" s="1"/>
-      <c r="R68" s="1"/>
-      <c r="S68" s="1"/>
+      <c r="R68" s="18"/>
+      <c r="S68" s="18"/>
       <c r="T68" s="1"/>
       <c r="U68" s="1"/>
       <c r="V68" s="1"/>
@@ -3866,14 +3249,10 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="13">
-      <c r="A69" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="C69" s="1"/>
-      <c r="D69" s="1"/>
+      <c r="A69" s="18"/>
+      <c r="B69" s="18"/>
+      <c r="C69" s="18"/>
+      <c r="D69" s="18"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
@@ -3887,8 +3266,8 @@
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
       <c r="Q69" s="1"/>
-      <c r="R69" s="1"/>
-      <c r="S69" s="1"/>
+      <c r="R69" s="18"/>
+      <c r="S69" s="18"/>
       <c r="T69" s="1"/>
       <c r="U69" s="1"/>
       <c r="V69" s="1"/>
@@ -3898,23 +3277,13 @@
       <c r="Z69" s="1"/>
     </row>
     <row r="70" spans="1:26" ht="13">
-      <c r="A70" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="D70" s="19" t="s">
-        <v>193</v>
-      </c>
+      <c r="A70" s="18"/>
+      <c r="B70" s="18"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="18"/>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
-      <c r="G70" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G70" s="1"/>
       <c r="H70" s="1"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
@@ -3936,23 +3305,13 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="13">
-      <c r="A71" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="C71" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="D71" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="E71" s="19" t="s">
-        <v>65</v>
-      </c>
+      <c r="A71" s="18"/>
+      <c r="B71" s="18"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
       <c r="F71" s="1"/>
-      <c r="G71" s="19"/>
+      <c r="G71" s="1"/>
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
@@ -3974,27 +3333,17 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="13">
-      <c r="A72" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C72" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="D72" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="E72" s="7" t="s">
-        <v>65</v>
-      </c>
+      <c r="A72" s="18"/>
+      <c r="B72" s="18"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="1"/>
       <c r="F72" s="1"/>
-      <c r="G72" s="19"/>
+      <c r="G72" s="18"/>
       <c r="H72" s="1"/>
-      <c r="I72" s="7"/>
-      <c r="J72" s="25"/>
-      <c r="K72" s="25"/>
+      <c r="I72" s="1"/>
+      <c r="J72" s="1"/>
+      <c r="K72" s="1"/>
       <c r="L72" s="1"/>
       <c r="M72" s="1"/>
       <c r="N72" s="1"/>
@@ -4012,21 +3361,13 @@
       <c r="Z72" s="1"/>
     </row>
     <row r="73" spans="1:26" ht="13">
-      <c r="A73" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B73" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="C73" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="E73" s="1"/>
+      <c r="A73" s="18"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="18"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="18"/>
       <c r="F73" s="1"/>
-      <c r="G73" s="19"/>
+      <c r="G73" s="18"/>
       <c r="H73" s="1"/>
       <c r="I73" s="1"/>
       <c r="J73" s="1"/>
@@ -4048,21 +3389,17 @@
       <c r="Z73" s="1"/>
     </row>
     <row r="74" spans="1:26" ht="13">
-      <c r="A74" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B74" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C74" s="19"/>
-      <c r="D74" s="19"/>
-      <c r="E74" s="1"/>
+      <c r="A74" s="7"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="18"/>
+      <c r="D74" s="7"/>
+      <c r="E74" s="7"/>
       <c r="F74" s="1"/>
-      <c r="G74" s="19"/>
+      <c r="G74" s="18"/>
       <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1"/>
-      <c r="K74" s="1"/>
+      <c r="I74" s="7"/>
+      <c r="J74" s="24"/>
+      <c r="K74" s="24"/>
       <c r="L74" s="1"/>
       <c r="M74" s="1"/>
       <c r="N74" s="1"/>
@@ -4080,23 +3417,13 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="13">
-      <c r="A75" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B75" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="C75" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="D75" s="19" t="s">
-        <v>206</v>
-      </c>
+      <c r="A75" s="7"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
-      <c r="G75" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G75" s="18"/>
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
@@ -4118,33 +3445,17 @@
       <c r="Z75" s="1"/>
     </row>
     <row r="76" spans="1:26" ht="13">
-      <c r="A76" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="B76" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="C76" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="D76" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="E76" s="19" t="s">
-        <v>65</v>
-      </c>
+      <c r="A76" s="7"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="18"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="1"/>
       <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
+      <c r="G76" s="18"/>
       <c r="H76" s="1"/>
-      <c r="I76" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="J76" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="K76" s="23" t="s">
-        <v>213</v>
-      </c>
+      <c r="I76" s="1"/>
+      <c r="J76" s="1"/>
+      <c r="K76" s="1"/>
       <c r="L76" s="1"/>
       <c r="M76" s="1"/>
       <c r="N76" s="1"/>
@@ -4162,23 +3473,13 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="13">
-      <c r="A77" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B77" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="C77" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="D77" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E77" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="F77" s="19"/>
-      <c r="G77" s="1"/>
+      <c r="A77" s="18"/>
+      <c r="B77" s="18"/>
+      <c r="C77" s="18"/>
+      <c r="D77" s="18"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="18"/>
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
@@ -4200,25 +3501,17 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="13">
-      <c r="A78" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B78" s="19" t="s">
-        <v>217</v>
-      </c>
-      <c r="C78" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="D78" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="E78" s="1"/>
+      <c r="A78" s="18"/>
+      <c r="B78" s="18"/>
+      <c r="C78" s="18"/>
+      <c r="D78" s="18"/>
+      <c r="E78" s="18"/>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
-      <c r="I78" s="1"/>
-      <c r="J78" s="1"/>
-      <c r="K78" s="1"/>
+      <c r="I78" s="18"/>
+      <c r="J78" s="22"/>
+      <c r="K78" s="22"/>
       <c r="L78" s="1"/>
       <c r="M78" s="1"/>
       <c r="N78" s="1"/>
@@ -4236,17 +3529,13 @@
       <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="13">
-      <c r="A79" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B79" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="C79" s="19"/>
-      <c r="D79" s="19"/>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="19"/>
+      <c r="A79" s="18"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="18"/>
+      <c r="G79" s="1"/>
       <c r="H79" s="1"/>
       <c r="I79" s="1"/>
       <c r="J79" s="1"/>
@@ -4268,23 +3557,13 @@
       <c r="Z79" s="1"/>
     </row>
     <row r="80" spans="1:26" ht="13">
-      <c r="A80" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="B80" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="C80" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="D80" s="19" t="s">
-        <v>222</v>
-      </c>
+      <c r="A80" s="18"/>
+      <c r="B80" s="18"/>
+      <c r="C80" s="18"/>
+      <c r="D80" s="18"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
-      <c r="G80" s="19" t="s">
-        <v>48</v>
-      </c>
+      <c r="G80" s="1"/>
       <c r="H80" s="1"/>
       <c r="I80" s="1"/>
       <c r="J80" s="1"/>
@@ -4306,23 +3585,13 @@
       <c r="Z80" s="1"/>
     </row>
     <row r="81" spans="1:26" ht="13">
-      <c r="A81" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="B81" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="C81" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="D81" s="19" t="s">
-        <v>225</v>
-      </c>
-      <c r="E81" s="19" t="s">
-        <v>65</v>
-      </c>
+      <c r="A81" s="18"/>
+      <c r="B81" s="18"/>
+      <c r="C81" s="18"/>
+      <c r="D81" s="18"/>
+      <c r="E81" s="1"/>
       <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
+      <c r="G81" s="18"/>
       <c r="H81" s="1"/>
       <c r="I81" s="1"/>
       <c r="J81" s="1"/>
@@ -4344,23 +3613,13 @@
       <c r="Z81" s="1"/>
     </row>
     <row r="82" spans="1:26" ht="13">
-      <c r="A82" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B82" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="C82" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="D82" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="E82" s="19" t="s">
-        <v>65</v>
-      </c>
+      <c r="A82" s="18"/>
+      <c r="B82" s="18"/>
+      <c r="C82" s="18"/>
+      <c r="D82" s="18"/>
+      <c r="E82" s="1"/>
       <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
+      <c r="G82" s="18"/>
       <c r="H82" s="1"/>
       <c r="I82" s="1"/>
       <c r="J82" s="1"/>
@@ -4382,19 +3641,11 @@
       <c r="Z82" s="1"/>
     </row>
     <row r="83" spans="1:26" ht="13">
-      <c r="A83" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B83" s="19" t="s">
-        <v>229</v>
-      </c>
-      <c r="C83" s="19" t="s">
-        <v>230</v>
-      </c>
-      <c r="D83" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="E83" s="1"/>
+      <c r="A83" s="18"/>
+      <c r="B83" s="18"/>
+      <c r="C83" s="18"/>
+      <c r="D83" s="18"/>
+      <c r="E83" s="18"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
       <c r="H83" s="1"/>
@@ -4418,15 +3669,11 @@
       <c r="Z83" s="1"/>
     </row>
     <row r="84" spans="1:26" ht="13">
-      <c r="A84" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B84" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="C84" s="1"/>
-      <c r="D84" s="1"/>
-      <c r="E84" s="1"/>
+      <c r="A84" s="18"/>
+      <c r="B84" s="18"/>
+      <c r="C84" s="18"/>
+      <c r="D84" s="18"/>
+      <c r="E84" s="18"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
@@ -4450,10 +3697,10 @@
       <c r="Z84" s="1"/>
     </row>
     <row r="85" spans="1:26" ht="13">
-      <c r="A85" s="1"/>
-      <c r="B85" s="1"/>
-      <c r="C85" s="1"/>
-      <c r="D85" s="1"/>
+      <c r="A85" s="18"/>
+      <c r="B85" s="18"/>
+      <c r="C85" s="18"/>
+      <c r="D85" s="18"/>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
@@ -4478,8 +3725,8 @@
       <c r="Z85" s="1"/>
     </row>
     <row r="86" spans="1:26" ht="13">
-      <c r="A86" s="1"/>
-      <c r="B86" s="1"/>
+      <c r="A86" s="18"/>
+      <c r="B86" s="18"/>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
       <c r="E86" s="1"/>
@@ -31021,39 +30268,95 @@
       <c r="Y1033" s="1"/>
       <c r="Z1033" s="1"/>
     </row>
+    <row r="1034" spans="1:26" ht="13">
+      <c r="A1034" s="1"/>
+      <c r="B1034" s="1"/>
+      <c r="C1034" s="1"/>
+      <c r="D1034" s="1"/>
+      <c r="E1034" s="1"/>
+      <c r="F1034" s="1"/>
+      <c r="G1034" s="1"/>
+      <c r="H1034" s="1"/>
+      <c r="I1034" s="1"/>
+      <c r="J1034" s="1"/>
+      <c r="K1034" s="1"/>
+      <c r="L1034" s="1"/>
+      <c r="M1034" s="1"/>
+      <c r="N1034" s="1"/>
+      <c r="O1034" s="1"/>
+      <c r="P1034" s="1"/>
+      <c r="Q1034" s="1"/>
+      <c r="R1034" s="1"/>
+      <c r="S1034" s="1"/>
+      <c r="T1034" s="1"/>
+      <c r="U1034" s="1"/>
+      <c r="V1034" s="1"/>
+      <c r="W1034" s="1"/>
+      <c r="X1034" s="1"/>
+      <c r="Y1034" s="1"/>
+      <c r="Z1034" s="1"/>
+    </row>
+    <row r="1035" spans="1:26" ht="13">
+      <c r="A1035" s="1"/>
+      <c r="B1035" s="1"/>
+      <c r="C1035" s="1"/>
+      <c r="D1035" s="1"/>
+      <c r="E1035" s="1"/>
+      <c r="F1035" s="1"/>
+      <c r="G1035" s="1"/>
+      <c r="H1035" s="1"/>
+      <c r="I1035" s="1"/>
+      <c r="J1035" s="1"/>
+      <c r="K1035" s="1"/>
+      <c r="L1035" s="1"/>
+      <c r="M1035" s="1"/>
+      <c r="N1035" s="1"/>
+      <c r="O1035" s="1"/>
+      <c r="P1035" s="1"/>
+      <c r="Q1035" s="1"/>
+      <c r="R1035" s="1"/>
+      <c r="S1035" s="1"/>
+      <c r="T1035" s="1"/>
+      <c r="U1035" s="1"/>
+      <c r="V1035" s="1"/>
+      <c r="W1035" s="1"/>
+      <c r="X1035" s="1"/>
+      <c r="Y1035" s="1"/>
+      <c r="Z1035" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C41:D41"/>
+  <mergeCells count="1">
+    <mergeCell ref="C43:D43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z20"/>
+  <dimension ref="A1:Z34"/>
   <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15.40625" customWidth="1"/>
     <col min="2" max="2" width="18.26953125" customWidth="1"/>
     <col min="3" max="3" width="52.6796875" customWidth="1"/>
+    <col min="4" max="4" width="90.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
-      <c r="A1" s="26" t="s">
-        <v>232</v>
+    <row r="1" spans="1:26" ht="15.25">
+      <c r="A1" s="25" t="s">
+        <v>60</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1"/>
@@ -31080,278 +30383,445 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A2" s="28" t="s">
-        <v>233</v>
+      <c r="A2" s="27" t="s">
+        <v>61</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A3" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="28" t="s">
-        <v>234</v>
+      <c r="D3" s="27" t="s">
+        <v>66</v>
       </c>
-      <c r="D2" s="28" t="s">
-        <v>235</v>
+    </row>
+    <row r="4" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A4" s="27" t="s">
+        <v>55</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A3" s="28" t="s">
-        <v>233</v>
+      <c r="B4" s="27" t="s">
+        <v>67</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>236</v>
+      <c r="C4" s="27" t="s">
+        <v>68</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>237</v>
+      <c r="D4" s="27" t="s">
+        <v>69</v>
       </c>
-      <c r="D3" s="28" t="s">
-        <v>238</v>
+    </row>
+    <row r="5" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A5" s="27" t="s">
+        <v>55</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A4" s="28" t="s">
+      <c r="B5" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A6" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A7" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A8" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A9" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>239</v>
+      <c r="D9" s="27" t="s">
+        <v>82</v>
       </c>
-      <c r="C4" s="28" t="s">
-        <v>240</v>
+    </row>
+    <row r="10" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A10" s="27" t="s">
+        <v>59</v>
       </c>
-      <c r="D4" s="28" t="s">
-        <v>241</v>
+      <c r="B10" s="27" t="s">
+        <v>83</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="C10" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A11" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A12" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A13" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A14" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A15" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A16" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A17" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A18" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A19" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="13">
+      <c r="A20" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A21" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="D21" s="32" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A22" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A23" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A24" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B24" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A25" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B25" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A26" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A27" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A28" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="35" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A29" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" s="32" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A30" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B30" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="D30" s="34" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A31" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" s="34" t="s">
+        <v>183</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A32" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="C32" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="D32" s="33" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A33" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A34" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="C34" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>242</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A6" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>245</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A7" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A8" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>249</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>250</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A9" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>252</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>253</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A10" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>255</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>256</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A11" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B11" s="28" t="s">
-        <v>258</v>
-      </c>
-      <c r="C11" s="28" t="s">
-        <v>259</v>
-      </c>
-      <c r="D11" s="28" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A12" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B12" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A13" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>264</v>
-      </c>
-      <c r="C13" s="28" t="s">
-        <v>265</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A14" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>267</v>
-      </c>
-      <c r="C14" s="28" t="s">
-        <v>268</v>
-      </c>
-      <c r="D14" s="28" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A15" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>270</v>
-      </c>
-      <c r="C15" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A16" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B16" s="28" t="s">
-        <v>273</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>274</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A17" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>252</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>276</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A18" s="28" t="s">
-        <v>278</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>279</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>280</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A19" s="28" t="s">
-        <v>278</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>282</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>283</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="13">
-      <c r="A20" s="28" t="s">
-        <v>278</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>285</v>
-      </c>
-      <c r="C20" s="28" t="s">
-        <v>286</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>287</v>
+      <c r="D34" s="33" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -31360,22 +30830,22 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>288</v>
+        <v>116</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>289</v>
+        <v>117</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>290</v>
+        <v>118</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>291</v>
+        <v>119</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>292</v>
+        <v>120</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>293</v>
+        <v>121</v>
       </c>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -31399,20 +30869,20 @@
       <c r="Z1" s="3"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A2" s="21" t="s">
-        <v>294</v>
+      <c r="A2" s="20" t="s">
+        <v>122</v>
       </c>
-      <c r="B2" s="21" t="s">
-        <v>295</v>
+      <c r="B2" s="20" t="s">
+        <v>123</v>
       </c>
-      <c r="C2" s="30">
+      <c r="C2" s="29">
         <v>43596</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>296</v>
+        <v>124</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>297</v>
+        <v>125</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>

</xml_diff>